<commit_message>
Update board — 1 notes, 0 done (2026-08-17 14:38)
</commit_message>
<xml_diff>
--- a/todo-board.xlsx
+++ b/todo-board.xlsx
@@ -450,7 +450,7 @@
         <v>T-0HFNF28</v>
       </c>
       <c r="B2" t="str">
-        <v/>
+        <v xml:space="preserve">Coveo RSP </v>
       </c>
       <c r="C2" t="str">
         <v/>
@@ -565,7 +565,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E12"/>
   <cols>
     <col min="1" max="1" width="17.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -608,9 +608,179 @@
         <v/>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>2026-08-17 14:38</v>
+      </c>
+      <c r="B3" t="str">
+        <v>T-0HFNF28</v>
+      </c>
+      <c r="C3" t="str">
+        <v>C</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E3" t="str">
+        <v>C</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>2026-08-17 14:38</v>
+      </c>
+      <c r="B4" t="str">
+        <v>T-0HFNF28</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Co</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Co</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>2026-08-17 14:38</v>
+      </c>
+      <c r="B5" t="str">
+        <v>T-0HFNF28</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Cov</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Cov</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>2026-08-17 14:38</v>
+      </c>
+      <c r="B6" t="str">
+        <v>T-0HFNF28</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Cove</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Cove</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>2026-08-17 14:38</v>
+      </c>
+      <c r="B7" t="str">
+        <v>T-0HFNF28</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Coveo</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Coveo</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>2026-08-17 14:38</v>
+      </c>
+      <c r="B8" t="str">
+        <v>T-0HFNF28</v>
+      </c>
+      <c r="C8" t="str">
+        <v xml:space="preserve">Coveo </v>
+      </c>
+      <c r="D8" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E8" t="str">
+        <v xml:space="preserve">Coveo </v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>2026-08-17 14:38</v>
+      </c>
+      <c r="B9" t="str">
+        <v>T-0HFNF28</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Coveo R</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Coveo R</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>2026-08-17 14:38</v>
+      </c>
+      <c r="B10" t="str">
+        <v>T-0HFNF28</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Coveo RS</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Coveo RS</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>2026-08-17 14:38</v>
+      </c>
+      <c r="B11" t="str">
+        <v>T-0HFNF28</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Coveo RSP</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Coveo RSP</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>2026-08-17 14:38</v>
+      </c>
+      <c r="B12" t="str">
+        <v>T-0HFNF28</v>
+      </c>
+      <c r="C12" t="str">
+        <v xml:space="preserve">Coveo RSP </v>
+      </c>
+      <c r="D12" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E12" t="str">
+        <v xml:space="preserve">Coveo RSP </v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E12"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update board — 1 notes, 0 done (2026-08-17 14:39)
</commit_message>
<xml_diff>
--- a/todo-board.xlsx
+++ b/todo-board.xlsx
@@ -450,13 +450,13 @@
         <v>T-0HFNF28</v>
       </c>
       <c r="B2" t="str">
-        <v xml:space="preserve">Coveo RSP </v>
+        <v>Coveo RSP QPM Mail</v>
       </c>
       <c r="C2" t="str">
         <v/>
       </c>
       <c r="D2" t="str">
-        <v>To do</v>
+        <v>In progress</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -471,7 +471,7 @@
         <v/>
       </c>
       <c r="I2" t="str">
-        <v>2026-08-17 14:38</v>
+        <v>2026-08-17 14:39</v>
       </c>
       <c r="J2" t="str">
         <v>--p1</v>
@@ -513,7 +513,7 @@
         <v>To do</v>
       </c>
       <c r="B3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -521,7 +521,7 @@
         <v>In progress</v>
       </c>
       <c r="B4">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -553,7 +553,7 @@
         <v>Last saved</v>
       </c>
       <c r="B8" t="str">
-        <v>2026-08-17 14:38</v>
+        <v>2026-08-17 14:39</v>
       </c>
     </row>
   </sheetData>
@@ -565,7 +565,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E29"/>
   <cols>
     <col min="1" max="1" width="17.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -778,9 +778,298 @@
         <v xml:space="preserve">Coveo RSP </v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>2026-08-17 14:39</v>
+      </c>
+      <c r="B13" t="str">
+        <v>T-0HFNF28</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Coveo RSP Q</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Coveo RSP Q</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>2026-08-17 14:39</v>
+      </c>
+      <c r="B14" t="str">
+        <v>T-0HFNF28</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Coveo RSP QP</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Coveo RSP QP</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>2026-08-17 14:39</v>
+      </c>
+      <c r="B15" t="str">
+        <v>T-0HFNF28</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Coveo RSP QPM</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Coveo RSP QPM</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>2026-08-17 14:39</v>
+      </c>
+      <c r="B16" t="str">
+        <v>T-0HFNF28</v>
+      </c>
+      <c r="C16" t="str">
+        <v xml:space="preserve">Coveo RSP QPM </v>
+      </c>
+      <c r="D16" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E16" t="str">
+        <v xml:space="preserve">Coveo RSP QPM </v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>2026-08-17 14:39</v>
+      </c>
+      <c r="B17" t="str">
+        <v>T-0HFNF28</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Coveo RSP QPM M</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E17" t="str">
+        <v>Coveo RSP QPM M</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>2026-08-17 14:39</v>
+      </c>
+      <c r="B18" t="str">
+        <v>T-0HFNF28</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Coveo RSP QPM MA</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E18" t="str">
+        <v>Coveo RSP QPM MA</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>2026-08-17 14:39</v>
+      </c>
+      <c r="B19" t="str">
+        <v>T-0HFNF28</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Coveo RSP QPM MAi</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E19" t="str">
+        <v>Coveo RSP QPM MAi</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>2026-08-17 14:39</v>
+      </c>
+      <c r="B20" t="str">
+        <v>T-0HFNF28</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Coveo RSP QPM MAil</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E20" t="str">
+        <v>Coveo RSP QPM MAil</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>2026-08-17 14:39</v>
+      </c>
+      <c r="B21" t="str">
+        <v>T-0HFNF28</v>
+      </c>
+      <c r="C21" t="str">
+        <v xml:space="preserve">Coveo RSP QPM MAil </v>
+      </c>
+      <c r="D21" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E21" t="str">
+        <v xml:space="preserve">Coveo RSP QPM MAil </v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>2026-08-17 14:39</v>
+      </c>
+      <c r="B22" t="str">
+        <v>T-0HFNF28</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Coveo RSP QPM MAil</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E22" t="str">
+        <v>Coveo RSP QPM MAil</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>2026-08-17 14:39</v>
+      </c>
+      <c r="B23" t="str">
+        <v>T-0HFNF28</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Coveo RSP QPM MAi</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E23" t="str">
+        <v>Coveo RSP QPM MAi</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>2026-08-17 14:39</v>
+      </c>
+      <c r="B24" t="str">
+        <v>T-0HFNF28</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Coveo RSP QPM MA</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E24" t="str">
+        <v>Coveo RSP QPM MA</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>2026-08-17 14:39</v>
+      </c>
+      <c r="B25" t="str">
+        <v>T-0HFNF28</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Coveo RSP QPM M</v>
+      </c>
+      <c r="D25" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E25" t="str">
+        <v>Coveo RSP QPM M</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>2026-08-17 14:39</v>
+      </c>
+      <c r="B26" t="str">
+        <v>T-0HFNF28</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Coveo RSP QPM Ma</v>
+      </c>
+      <c r="D26" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E26" t="str">
+        <v>Coveo RSP QPM Ma</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>2026-08-17 14:39</v>
+      </c>
+      <c r="B27" t="str">
+        <v>T-0HFNF28</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Coveo RSP QPM Mai</v>
+      </c>
+      <c r="D27" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E27" t="str">
+        <v>Coveo RSP QPM Mai</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>2026-08-17 14:39</v>
+      </c>
+      <c r="B28" t="str">
+        <v>T-0HFNF28</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Coveo RSP QPM Mail</v>
+      </c>
+      <c r="D28" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E28" t="str">
+        <v>Coveo RSP QPM Mail</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>2026-08-17 14:39</v>
+      </c>
+      <c r="B29" t="str">
+        <v>T-0HFNF28</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Coveo RSP QPM Mail</v>
+      </c>
+      <c r="D29" t="str">
+        <v>Status changed</v>
+      </c>
+      <c r="E29" t="str">
+        <v>To do → In progress</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E29"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>